<commit_message>
Add FastAPI backend for mobile app integration
</commit_message>
<xml_diff>
--- a/outputs/sensitivity_000001_双均线策略.xlsx
+++ b/outputs/sensitivity_000001_双均线策略.xlsx
@@ -478,22 +478,22 @@
         <v>60</v>
       </c>
       <c r="C2" t="n">
-        <v>0.2290377180000001</v>
+        <v>0.2434158209999999</v>
       </c>
       <c r="D2" t="n">
-        <v>0.1139916501055791</v>
+        <v>0.2957562318769218</v>
       </c>
       <c r="E2" t="n">
-        <v>0.03496946101619924</v>
+        <v>0.04453567585820251</v>
       </c>
       <c r="F2" t="n">
-        <v>-0.3357693901803993</v>
+        <v>-0.3353744517939653</v>
       </c>
       <c r="G2" t="n">
-        <v>0.1816755116680701</v>
+        <v>0.224250972952973</v>
       </c>
       <c r="H2" t="n">
-        <v>18</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -504,22 +504,22 @@
         <v>60</v>
       </c>
       <c r="C3" t="n">
-        <v>0.05950343400000002</v>
+        <v>0.0888955520000001</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.05554263389442093</v>
+        <v>0.141235962876922</v>
       </c>
       <c r="E3" t="n">
-        <v>0.009679940439487167</v>
+        <v>0.01717867049094068</v>
       </c>
       <c r="F3" t="n">
-        <v>-0.3189560623721434</v>
+        <v>-0.318141923206567</v>
       </c>
       <c r="G3" t="n">
-        <v>0.06844306833414215</v>
+        <v>0.1108716798711266</v>
       </c>
       <c r="H3" t="n">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
@@ -530,22 +530,22 @@
         <v>60</v>
       </c>
       <c r="C4" t="n">
-        <v>0.05722758299999997</v>
+        <v>0.04841323399999986</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.05781848489442099</v>
+        <v>0.1007536448769217</v>
       </c>
       <c r="E4" t="n">
-        <v>0.009318145097482633</v>
+        <v>0.009500408156742912</v>
       </c>
       <c r="F4" t="n">
-        <v>-0.3883741261922881</v>
+        <v>-0.3880092103900082</v>
       </c>
       <c r="G4" t="n">
-        <v>0.06614167527167625</v>
+        <v>0.07735087207408249</v>
       </c>
       <c r="H4" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -556,22 +556,22 @@
         <v>60</v>
       </c>
       <c r="C5" t="n">
-        <v>-0.005052111999999997</v>
+        <v>0.02832727299999993</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.120098179894421</v>
+        <v>0.0806676838769218</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.0008437966472981673</v>
+        <v>0.005602329746093648</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.4470333469929385</v>
+        <v>-0.4452503924479221</v>
       </c>
       <c r="G5" t="n">
-        <v>0.02718632394767214</v>
+        <v>0.06784066824626954</v>
       </c>
       <c r="H5" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
@@ -582,22 +582,22 @@
         <v>15</v>
       </c>
       <c r="C6" t="n">
-        <v>-0.165533334</v>
+        <v>-0.226703874</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.280579401894421</v>
+        <v>-0.1743634631230782</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.02971012662055506</v>
+        <v>-0.05011907411365291</v>
       </c>
       <c r="F6" t="n">
-        <v>-0.5508986314594047</v>
+        <v>-0.5477503053531967</v>
       </c>
       <c r="G6" t="n">
-        <v>-0.09947080562649098</v>
+        <v>-0.1633327153079103</v>
       </c>
       <c r="H6" t="n">
-        <v>69</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7">
@@ -608,74 +608,74 @@
         <v>30</v>
       </c>
       <c r="C7" t="n">
-        <v>-0.250651761</v>
+        <v>-0.312948872</v>
       </c>
       <c r="D7" t="n">
-        <v>-0.3656978288944209</v>
+        <v>-0.2606084611230781</v>
       </c>
       <c r="E7" t="n">
-        <v>-0.04695381220639505</v>
+        <v>-0.07232081657318123</v>
       </c>
       <c r="F7" t="n">
-        <v>-0.5430981411164358</v>
+        <v>-0.5418206793932063</v>
       </c>
       <c r="G7" t="n">
-        <v>-0.175208434963275</v>
+        <v>-0.2560488564726752</v>
       </c>
       <c r="H7" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="B8" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C8" t="n">
-        <v>-0.2954386130000001</v>
+        <v>-0.373087592</v>
       </c>
       <c r="D8" t="n">
-        <v>-0.410484680894421</v>
+        <v>-0.3207471811230781</v>
       </c>
       <c r="E8" t="n">
-        <v>-0.05669282081892457</v>
+        <v>-0.08916151320625743</v>
       </c>
       <c r="F8" t="n">
-        <v>-0.5790996321788018</v>
+        <v>-0.5184088397637552</v>
       </c>
       <c r="G8" t="n">
-        <v>-0.234771726949503</v>
+        <v>-0.3761320109144147</v>
       </c>
       <c r="H8" t="n">
-        <v>43</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B9" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="C9" t="n">
-        <v>-0.342407049</v>
+        <v>-0.373949622</v>
       </c>
       <c r="D9" t="n">
-        <v>-0.4574531168944209</v>
+        <v>-0.3216092111230782</v>
       </c>
       <c r="E9" t="n">
-        <v>-0.06747705863175379</v>
+        <v>-0.08941213906839729</v>
       </c>
       <c r="F9" t="n">
-        <v>-0.6087146784010486</v>
+        <v>-0.5774222136928155</v>
       </c>
       <c r="G9" t="n">
-        <v>-0.2935261276591465</v>
+        <v>-0.3521042143934023</v>
       </c>
       <c r="H9" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10">
@@ -683,74 +683,74 @@
         <v>5</v>
       </c>
       <c r="B10" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="C10" t="n">
-        <v>-0.365120001</v>
+        <v>-0.395769029</v>
       </c>
       <c r="D10" t="n">
-        <v>-0.4801660688944209</v>
+        <v>-0.3434286181230781</v>
       </c>
       <c r="E10" t="n">
-        <v>-0.07292413668571718</v>
+        <v>-0.09584977144365958</v>
       </c>
       <c r="F10" t="n">
-        <v>-0.6370178940052689</v>
+        <v>-0.6077125190454304</v>
       </c>
       <c r="G10" t="n">
-        <v>-0.3003757186790703</v>
+        <v>-0.3902945911878181</v>
       </c>
       <c r="H10" t="n">
-        <v>62</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B11" t="n">
         <v>30</v>
       </c>
       <c r="C11" t="n">
-        <v>-0.37385514</v>
+        <v>-0.408886982</v>
       </c>
       <c r="D11" t="n">
-        <v>-0.4889012078944209</v>
+        <v>-0.3565465711230781</v>
       </c>
       <c r="E11" t="n">
-        <v>-0.07506232441308536</v>
+        <v>-0.09981016453858016</v>
       </c>
       <c r="F11" t="n">
-        <v>-0.5193709097168749</v>
+        <v>-0.622676998857518</v>
       </c>
       <c r="G11" t="n">
-        <v>-0.3455212520761114</v>
+        <v>-0.4220369631618129</v>
       </c>
       <c r="H11" t="n">
-        <v>27</v>
+        <v>25</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B12" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C12" t="n">
-        <v>-0.376951385</v>
+        <v>-0.412390316</v>
       </c>
       <c r="D12" t="n">
-        <v>-0.491997452894421</v>
+        <v>-0.3600499051230781</v>
       </c>
       <c r="E12" t="n">
-        <v>-0.07582619242038791</v>
+        <v>-0.1008797294293142</v>
       </c>
       <c r="F12" t="n">
-        <v>-0.6329662655084451</v>
+        <v>-0.6348322553242094</v>
       </c>
       <c r="G12" t="n">
-        <v>-0.3180113767209705</v>
+        <v>-0.3895780743037417</v>
       </c>
       <c r="H12" t="n">
         <v>52</v>
@@ -761,103 +761,103 @@
         <v>8</v>
       </c>
       <c r="B13" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="C13" t="n">
-        <v>-0.392674535</v>
+        <v>-0.4323008269999999</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.507720602894421</v>
+        <v>-0.3799604161230781</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.07975475539792976</v>
+        <v>-0.1070571742866422</v>
       </c>
       <c r="F13" t="n">
-        <v>-0.6235092751869733</v>
+        <v>-0.6007152091534591</v>
       </c>
       <c r="G13" t="n">
-        <v>-0.364638235476663</v>
+        <v>-0.4450488283751602</v>
       </c>
       <c r="H13" t="n">
-        <v>28</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B14" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C14" t="n">
-        <v>-0.423882345</v>
+        <v>-0.4374681070000001</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.5389284128944209</v>
+        <v>-0.3851276961230782</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.08781023007786237</v>
+        <v>-0.1086886641279583</v>
       </c>
       <c r="F14" t="n">
-        <v>-0.602772147522576</v>
+        <v>-0.6311252511498059</v>
       </c>
       <c r="G14" t="n">
-        <v>-0.3959760484608238</v>
+        <v>-0.4304377481211516</v>
       </c>
       <c r="H14" t="n">
-        <v>54</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B15" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C15" t="n">
-        <v>-0.443958549</v>
+        <v>-0.465095134</v>
       </c>
       <c r="D15" t="n">
-        <v>-0.5590046168944209</v>
+        <v>-0.4127547231230781</v>
       </c>
       <c r="E15" t="n">
-        <v>-0.09318674146837025</v>
+        <v>-0.1176207031985314</v>
       </c>
       <c r="F15" t="n">
-        <v>-0.5735351674313001</v>
+        <v>-0.6297944833765627</v>
       </c>
       <c r="G15" t="n">
-        <v>-0.419084945522249</v>
+        <v>-0.4985903898546761</v>
       </c>
       <c r="H15" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B16" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="C16" t="n">
-        <v>-0.447365682</v>
+        <v>-0.494020096</v>
       </c>
       <c r="D16" t="n">
-        <v>-0.562411749894421</v>
+        <v>-0.4416796851230781</v>
       </c>
       <c r="E16" t="n">
-        <v>-0.09411519480396768</v>
+        <v>-0.1273770039706292</v>
       </c>
       <c r="F16" t="n">
-        <v>-0.6316363280849546</v>
+        <v>-0.5721054968075915</v>
       </c>
       <c r="G16" t="n">
-        <v>-0.4297807979181703</v>
+        <v>-0.5394532090424011</v>
       </c>
       <c r="H16" t="n">
-        <v>54</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17">
@@ -868,22 +868,22 @@
         <v>20</v>
       </c>
       <c r="C17" t="n">
-        <v>-0.4801489609999999</v>
+        <v>-0.516032431</v>
       </c>
       <c r="D17" t="n">
-        <v>-0.5951950288944209</v>
+        <v>-0.4636920201230781</v>
       </c>
       <c r="E17" t="n">
-        <v>-0.1033014116680027</v>
+        <v>-0.1351052676332805</v>
       </c>
       <c r="F17" t="n">
-        <v>-0.5908894553622213</v>
+        <v>-0.5585821172683711</v>
       </c>
       <c r="G17" t="n">
-        <v>-0.4730788040881611</v>
+        <v>-0.5807579259935551</v>
       </c>
       <c r="H17" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>